<commit_message>
Bring the field spec's Calls sheet in line with the calls model; add member_id
The Calls sheet described an earlier design (provider_call_id, status enum,
turn-array transcript, collected_data). Rewrite it to match CallOut field for
field, and list member_id on the Patients sheet next to patient_id.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/patient_field_spec.xlsx
+++ b/docs/patient_field_spec.xlsx
@@ -42,7 +42,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +73,16 @@
         <bgColor rgb="00EAEAEA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAEAEA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4EA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -100,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -118,6 +128,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -485,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -937,20 +953,42 @@
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>member_id</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>8 random digits, unique (indexed). Read to the caller at registration; with full name + DOB, it verifies identity on later calls. Not in original spec table.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>deleted_at</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Soft-delete marker (UTC); null for active records. Set by DELETE /patients/:id — not in original spec table but required by the API contract.</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
@@ -967,7 +1005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1006,15 +1044,15 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>UUID</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Auto-generated unique identifier (primary key)</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+          <t>Retell's call ID; primary key (unique index). Tool calls and the webhook both key on it.</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
@@ -1023,20 +1061,20 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>patient_id</t>
+          <t>from_number</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>UUID (FK)</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>FK → patients.patient_id. Null if the call ended before any record was created; points at the existing patient on an update call.</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
+          <t>Caller's number as Retell reports it. Duplicate detection runs on patients (phone + name + DOB), not here.</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1045,7 +1083,7 @@
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>phone_number</t>
+          <t>to_number</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1055,19 +1093,19 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Caller's number, U.S. 10-digit. Indexed — used for returning-caller / duplicate detection before a patient_id exists.</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Number the caller dialed.</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>provider_call_id</t>
+          <t>direction</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1077,10 +1115,10 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Telephony provider's call SID (Vapi / Retell / Twilio). For cross-referencing their dashboard and recordings.</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+          <t>inbound or outbound, as Retell reports it.</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1094,59 +1132,59 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Enum</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>in_progress, completed_registration, completed_update, abandoned, error</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Retell's call_status as sent: registered, ongoing, ended, error.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>transcript</t>
+          <t>started_at</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>Timestamp</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Array of turns: [{ role, text, ts }]. Structured rather than a flat blob so corrections can be inspected turn-by-turn.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Call start (UTC), from Retell's start_timestamp.</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>collected_data</t>
+          <t>ended_at</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>Timestamp</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Snapshot of final slot values sent to POST /patients. Satisfies the observability requirement structurally.</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
+          <t>Call end (UTC), from Retell's end_timestamp. Null while the call is live.</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1155,20 +1193,20 @@
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>error_message</t>
+          <t>duration_ms</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Populated when status = error (e.g. DB write failure); null otherwise.</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
+          <t>end_timestamp − start_timestamp. Both are provider timestamps, so no local clock is involved.</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1177,42 +1215,42 @@
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>started_at</t>
+          <t>disconnection_reason</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Call start (UTC)</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Retell's reason the call ended (e.g. user_hangup, agent_hangup).</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ended_at</t>
+          <t>transcript</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Call end (UTC). Null while status = in_progress.</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
+          <t>Plain-text transcript from the call_ended webhook. The full webhook body is kept in the logs collection (90 days).</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1221,20 +1259,20 @@
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>duration_seconds</t>
+          <t>recording_url</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Taken from the provider's end-of-call webhook rather than computed locally (avoids webhook clock drift).</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
+          <t>Retell-hosted call recording.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1243,20 +1281,108 @@
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>call_analysis</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Retell's post-call analysis (e.g. summary, sentiment), from the call_analyzed webhook.</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>verified_patient_id</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>UUID (FK)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>FK → patients.patient_id. Set by verify_patient on a match; required to read or update a profile on this call.</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>verified_at</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Auto-generated at row insert (UTC)</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>When verification succeeded (UTC). Null if the caller never verified.</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>verification_attempts</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Number of verify_patient calls made on this call. Defaults to 0.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>patients_created</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Array (UUID FK)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>patient_ids registered on this call (FK → patients.patient_id). Defaults to [].</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>

</xml_diff>